<commit_message>
Add leads summary sheet
Co-authored-by: smbehm <smbehm@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/bali_leads_FULL.xlsx
+++ b/bali_leads_FULL.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet name="ALL leads" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="NO website only" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary by niche" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ALL leads'!$A$1:$H$336</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NO website only'!$A$1:$H$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary by niche'!$A$1:$D$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,13 +23,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -50,8 +55,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -782,7 +788,6 @@
           <t>https://wa.me/6287861615259</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1188,8 +1193,6 @@
           <t>QuitoArtBali Woodworking Project</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Jl. Subita Gg. VII No.4, Sumerta Kaja, Kec. Denpasar Tim., Kota Denpasar, Bali 80237, Indonesia</t>
@@ -2230,8 +2233,6 @@
           <t>tukang listrik panggilan cepat badung denpasar tabanan 24jam</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Dalung, Kec. Kuta Utara, denpasar kota, Bali 80113, Indonesia</t>
@@ -2642,8 +2643,6 @@
           <t>PT. Jaya Kusuma Sarana Bali (JKS Bali)</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Jl. Imam Bonjol No.555, Pemecutan Klod, Denpasar Barat, Denpasar City, Bali 80119, Indonesia</t>
@@ -2760,8 +2759,6 @@
           <t>BANDAR LAUNDRY EXPRESS</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Jl. Buana Raya, Padangsambian, Kec. Denpasar Bar., Kota Denpasar, Bali 80119, Indonesia</t>
@@ -3214,8 +3211,6 @@
           <t>Mama Laundry Kuta</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>Depan hotel Mertha Jati dan Bungalow, Jl. Kubu Anyar No.42, Kuta, Kec. Kuta, Kabupaten Badung, Bali 80361, Indonesia</t>
@@ -3710,8 +3705,6 @@
           <t>Laundry Express</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>8546+GW2, Jl. Camplung Tanduk, Seminyak, Kuta, Badung Regency, Bali 80361, Indonesia</t>
@@ -4626,8 +4619,6 @@
           <t>세탁소MaeMae Laundry</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>Jl. Monkey Forest, Ubud, Gianyar Regency, Bali 80751, Indonesia</t>
@@ -5542,8 +5533,6 @@
           <t>Cahaya Mulya</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>Jl. Gatot Subroto Tim. No.505, Kesiman Petilan, East Denpasar, Denpasar City, Bali 80237, Indonesia</t>
@@ -5828,8 +5817,6 @@
           <t>QuitoArtBali Woodworking Project</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>Jl. Subita Gg. VII No.4, Sumerta Kaja, Kec. Denpasar Tim., Kota Denpasar, Bali 80237, Indonesia</t>
@@ -6492,8 +6479,6 @@
           <t>tukang listrik panggilan cepat badung denpasar tabanan 24jam</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>Dalung, Kec. Kuta Utara, denpasar kota, Bali 80113, Indonesia</t>
@@ -7366,8 +7351,6 @@
           <t>CV. Made Carpenter Bali</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr"/>
-      <c r="C168" t="inlineStr"/>
       <c r="D168" t="inlineStr">
         <is>
           <t>98P4+JC9, Sukawati, Kec. Sukawati, Kabupaten Gianyar, Bali, Indonesia</t>
@@ -7652,8 +7635,6 @@
           <t>Bali Miracle Catering</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr"/>
-      <c r="C175" t="inlineStr"/>
       <c r="D175" t="inlineStr">
         <is>
           <t>Perumahan Puri Gading, Gg. Bendesa No.9, Jimbaran, South Kuta, Badung Regency, Bali 80361, Indonesia</t>
@@ -7938,8 +7919,6 @@
           <t>RG Bali Catering</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr"/>
-      <c r="C182" t="inlineStr"/>
       <c r="D182" t="inlineStr">
         <is>
           <t>Jl. Tegal Luwih XXV No.43-38, Dalung, Kec. Kuta Utara, Kabupaten Badung, Bali 80361, Indonesia</t>
@@ -8476,8 +8455,6 @@
           <t>Laundry Open Canggu</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr"/>
-      <c r="C195" t="inlineStr"/>
       <c r="D195" t="inlineStr">
         <is>
           <t>Jl. Raya Babakan Canggu No.35, Banjar Babakan, Canggu, Kuta Utara, Badung Regency, Bali 80361, Indonesia</t>
@@ -9024,7 +9001,6 @@
           <t>https://wa.me/6281239026015</t>
         </is>
       </c>
-      <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
           <t>YES</t>
@@ -9892,8 +9868,6 @@
           <t>Good Laundry Tukad Balian</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr"/>
       <c r="D229" t="inlineStr">
         <is>
           <t>Jl. Tukad Balian No.154, Renon, Denpasar Selatan, Denpasar City, Bali 80226, Indonesia</t>
@@ -11700,7 +11674,6 @@
           <t>https://wa.me/628123816525</t>
         </is>
       </c>
-      <c r="D272" t="inlineStr"/>
       <c r="E272" t="inlineStr">
         <is>
           <t>YES</t>
@@ -11948,7 +11921,6 @@
           <t>https://wa.me/6281338185304</t>
         </is>
       </c>
-      <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr">
         <is>
           <t>YES</t>
@@ -12438,8 +12410,6 @@
           <t>Service AC</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr"/>
-      <c r="C290" t="inlineStr"/>
       <c r="D290" t="inlineStr">
         <is>
           <t>jln Ratna perum Bayuh asri blok 3 no 75, Ungasan, Kec. Kuta Sel., Kabupaten Badung, Bali 80361, Indonesia</t>
@@ -12472,8 +12442,6 @@
           <t>Service Ac Di Bali</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr"/>
-      <c r="C291" t="inlineStr"/>
       <c r="D291" t="inlineStr">
         <is>
           <t>96GR+JCM, Jl. Trenggana, Penatih, Kec. Denpasar Tim., Kota Denpasar, Bali 80237, Indonesia</t>
@@ -13514,8 +13482,6 @@
           <t>RHEA florist &amp; Decorations Bali</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr"/>
-      <c r="C316" t="inlineStr"/>
       <c r="D316" t="inlineStr">
         <is>
           <t>kerobokan Jl. Intan Permai No.22 A, Kerobokan Kelod, Kec. Kuta Utara, Kabupaten Badung, Bali 80361, Indonesia</t>
@@ -13768,7 +13734,6 @@
           <t>https://wa.me/6282237810706</t>
         </is>
       </c>
-      <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
           <t>YES</t>
@@ -14755,7 +14720,6 @@
           <t>https://wa.me/6287861615259</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>NO</t>
@@ -15161,8 +15125,6 @@
           <t>QuitoArtBali Woodworking Project</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
           <t>Jl. Subita Gg. VII No.4, Sumerta Kaja, Kec. Denpasar Tim., Kota Denpasar, Bali 80237, Indonesia</t>
@@ -16203,8 +16165,6 @@
           <t>tukang listrik panggilan cepat badung denpasar tabanan 24jam</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
       <c r="D44" t="inlineStr">
         <is>
           <t>Dalung, Kec. Kuta Utara, denpasar kota, Bali 80113, Indonesia</t>
@@ -16615,8 +16575,6 @@
           <t>PT. Jaya Kusuma Sarana Bali (JKS Bali)</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
       <c r="D54" t="inlineStr">
         <is>
           <t>Jl. Imam Bonjol No.555, Pemecutan Klod, Denpasar Barat, Denpasar City, Bali 80119, Indonesia</t>
@@ -16733,8 +16691,6 @@
           <t>BANDAR LAUNDRY EXPRESS</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
       <c r="D57" t="inlineStr">
         <is>
           <t>Jl. Buana Raya, Padangsambian, Kec. Denpasar Bar., Kota Denpasar, Bali 80119, Indonesia</t>
@@ -17187,8 +17143,6 @@
           <t>Mama Laundry Kuta</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
       <c r="D68" t="inlineStr">
         <is>
           <t>Depan hotel Mertha Jati dan Bungalow, Jl. Kubu Anyar No.42, Kuta, Kec. Kuta, Kabupaten Badung, Bali 80361, Indonesia</t>
@@ -17683,8 +17637,6 @@
           <t>Laundry Express</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr">
         <is>
           <t>8546+GW2, Jl. Camplung Tanduk, Seminyak, Kuta, Badung Regency, Bali 80361, Indonesia</t>
@@ -18599,8 +18551,6 @@
           <t>세탁소MaeMae Laundry</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
-      <c r="C102" t="inlineStr"/>
       <c r="D102" t="inlineStr">
         <is>
           <t>Jl. Monkey Forest, Ubud, Gianyar Regency, Bali 80751, Indonesia</t>
@@ -19515,8 +19465,6 @@
           <t>Cahaya Mulya</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
-      <c r="C124" t="inlineStr"/>
       <c r="D124" t="inlineStr">
         <is>
           <t>Jl. Gatot Subroto Tim. No.505, Kesiman Petilan, East Denpasar, Denpasar City, Bali 80237, Indonesia</t>
@@ -19801,8 +19749,6 @@
           <t>QuitoArtBali Woodworking Project</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
-      <c r="C131" t="inlineStr"/>
       <c r="D131" t="inlineStr">
         <is>
           <t>Jl. Subita Gg. VII No.4, Sumerta Kaja, Kec. Denpasar Tim., Kota Denpasar, Bali 80237, Indonesia</t>
@@ -20465,8 +20411,6 @@
           <t>tukang listrik panggilan cepat badung denpasar tabanan 24jam</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
-      <c r="C147" t="inlineStr"/>
       <c r="D147" t="inlineStr">
         <is>
           <t>Dalung, Kec. Kuta Utara, denpasar kota, Bali 80113, Indonesia</t>
@@ -20917,4 +20861,383 @@
   <autoFilter ref="A1:H157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Search query / niche</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Total businesses</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>NO website</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>YES website</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>laundry Kuta Bali</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>18</v>
+      </c>
+      <c r="C2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>laundry Seminyak Bali</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>laundry Ubud Bali</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="n">
+        <v>13</v>
+      </c>
+      <c r="D4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tukang kayu Bali</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tukang listrik Bali</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>18</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AC service Bali</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>19</v>
+      </c>
+      <c r="C7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>carpenter Bali</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>14</v>
+      </c>
+      <c r="C8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>electrician Bali</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" t="n">
+        <v>9</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>renovasi villa Bali</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>17</v>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D10" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cleaning service Canggu Bali</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>20</v>
+      </c>
+      <c r="C11" t="n">
+        <v>8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>kontraktor Bali</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>20</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6</v>
+      </c>
+      <c r="D12" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>laundry Denpasar Bali</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>pest control Bali</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>20</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>catering Bali</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>20</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>jasa kebersihan Bali</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>wedding florist Bali</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>wedding organizer Bali</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>19</v>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>private driver Bali</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>20</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>service AC Bali</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>sopir pribadi Bali</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cleaning service Seminyak Bali</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D22"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>